<commit_message>
Aggiornato testbook frontend con esiti finali e screenshot
</commit_message>
<xml_diff>
--- a/docs/testbook/ClinicaFlow_TestBook_frontend.xlsx
+++ b/docs/testbook/ClinicaFlow_TestBook_frontend.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valen\clinicaflow\docs\testbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27DA7611-C18E-45BE-B3C8-C2DB0F73D40A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487B4771-213A-4A44-8D6E-C45D29B716E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{7DF372AB-F5E5-48F5-A7AF-34ACFEB5FD6C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="463" xr2:uid="{7DF372AB-F5E5-48F5-A7AF-34ACFEB5FD6C}"/>
   </bookViews>
   <sheets>
     <sheet name="ClinicaFlow_TestBook_frontend" sheetId="1" r:id="rId1"/>
+    <sheet name="TS1_20260403" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="177">
   <si>
     <t>ID Test</t>
   </si>
@@ -100,9 +101,6 @@
     <t>/api/patients/by-taxcode/{taxCode}</t>
   </si>
   <si>
-    <t>400 Bad Request</t>
-  </si>
-  <si>
     <t>PUT</t>
   </si>
   <si>
@@ -388,42 +386,12 @@
     <t>TCF23</t>
   </si>
   <si>
-    <t>Verificare il blocco della prenotazione su slot non disponibile dal Back Office.</t>
-  </si>
-  <si>
-    <t>{"patientId":&lt;ID_PATIENT&gt;,"availabilitySlotId":&lt;ID_SLOT_NON_DISPONIBILE&gt;,"notes":"Tentativo duplicato"}</t>
-  </si>
-  <si>
-    <t>Il sistema rifiuta la prenotazione perché lo slot selezionato non è più disponibile; il frontend mostra l'errore e la tabella non viene aggiornata.</t>
-  </si>
-  <si>
     <t>TCF24</t>
   </si>
   <si>
-    <t>MedicalReports</t>
-  </si>
-  <si>
-    <t>Verificare il blocco della creazione di un referto per appuntamento non completato dal Back Office.</t>
-  </si>
-  <si>
-    <t>{"appointmentId":&lt;ID_APPUNTAMENTO_SCHEDULED&gt;,"diagnosis":"Diagnosi errata","therapy":"Terapia errata","notes":"Test vincolo"}</t>
-  </si>
-  <si>
-    <t>Il sistema rifiuta la creazione del referto perché è consentita solo per appuntamenti completati; il frontend mostra l'errore senza creare il referto.</t>
-  </si>
-  <si>
     <t>TCF25</t>
   </si>
   <si>
-    <t>Verificare la creazione di un referto per appuntamento completato dal Back Office.</t>
-  </si>
-  <si>
-    <t>{"appointmentId":&lt;ID_APPUNTAMENTO_COMPLETATO&gt;,"diagnosis":"Visita di controllo","therapy":"Nessuna terapia","notes":"Referto creato da Back Office"}</t>
-  </si>
-  <si>
-    <t>Il referto viene creato correttamente e compare nella tabella referti del Back Office.</t>
-  </si>
-  <si>
     <t>Back Office</t>
   </si>
   <si>
@@ -478,24 +446,6 @@
     <t>TCF26</t>
   </si>
   <si>
-    <t>TCF27</t>
-  </si>
-  <si>
-    <t>TCF28</t>
-  </si>
-  <si>
-    <t>TCF29</t>
-  </si>
-  <si>
-    <t>TCF29_CreateReport_Completed_Success.png</t>
-  </si>
-  <si>
-    <t>TCF28_CreateReport_NotCompleted_BadRequest.png</t>
-  </si>
-  <si>
-    <t>TCF27_CreateAppointment_UnavailableSlot_Conflict.png</t>
-  </si>
-  <si>
     <t>TCF26_CreateAppointment_Success.png</t>
   </si>
   <si>
@@ -563,6 +513,45 @@
   </si>
   <si>
     <t>TCF20_CreatePatient_DuplicateTaxCode_Conflict.png</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>/api/doctors/by-taxcode/BNCLCU80A01H501Q</t>
+  </si>
+  <si>
+    <t>BNCLCU80A01H501Q</t>
+  </si>
+  <si>
+    <t>BNCLCU80A01H501R</t>
+  </si>
+  <si>
+    <t>/api/doctors/by-taxcode/BNCLCU80A01H501R</t>
+  </si>
+  <si>
+    <t>/api/appointments/9/status</t>
+  </si>
+  <si>
+    <t>/api/appointments/10/status</t>
+  </si>
+  <si>
+    <t>{"appointmentId":9,"diagnosis":"Diagnosi di test","therapy":"Terapia di test","notes":"Note di test"}</t>
+  </si>
+  <si>
+    <t>{"appointmentId":9,"diagnosis":"Diagnosi aggiornata","therapy":"Terapia aggiornata","notes":"Note aggiornate"}</t>
+  </si>
+  <si>
+    <t>{"firstName":"Giulia","lastName":"Neri","taxCode":"NREGLI85A41H501Z","specialtyId":8}</t>
+  </si>
+  <si>
+    <t>{"doctorId":9,"startTime":"2026-04-10T09:00:00","endTime":"2026-04-10T09:30:00"}</t>
+  </si>
+  <si>
+    <t>{"doctorId":9,"startTime":"2026-04-10T09:15:00","endTime":"2026-04-10T09:45:00"}</t>
+  </si>
+  <si>
+    <t>{"patientId":4,"availabilitySlotId":4,"notes":"Prenotazione da frontend"}</t>
   </si>
 </sst>
 </file>
@@ -1096,7 +1085,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="32">
     <dxf>
       <fill>
         <patternFill>
@@ -1110,6 +1099,62 @@
           <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1167,21 +1212,42 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A5FE12E1-30BD-4610-B2EA-DC3BCD910670}" name="Table134" displayName="Table134" ref="A1:L30" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
-  <autoFilter ref="A1:L30" xr:uid="{A5FE12E1-30BD-4610-B2EA-DC3BCD910670}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A5FE12E1-30BD-4610-B2EA-DC3BCD910670}" name="Table134" displayName="Table134" ref="A1:L27" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+  <autoFilter ref="A1:L27" xr:uid="{A5FE12E1-30BD-4610-B2EA-DC3BCD910670}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{EB876EC9-8950-4C9E-86BE-0FACA74E1014}" name="ID Test" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{EB9B5E9C-47F6-4F74-AAF0-EA51262287B5}" name="Area" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{52078D58-E160-4F5C-8E20-667269BD8E65}" name="Obiettivo" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{683810AF-1BE0-4D6F-9DB9-17FE773290C1}" name="Endpoint" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{9154901E-12A0-4767-BCFB-66395C70A786}" name="Metodo HTTP" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{C2F5DBF9-5AF1-4772-AC3D-C8C62175A99E}" name="Payload JSON" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{0E07DB66-29AC-4137-8446-4A4A24F26F1E}" name="Risultato atteso - Status Code" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{803671B0-E093-430D-967C-418EDDBE36A7}" name="Risultato atteso - Dettaglio" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{FB4642C7-35C4-4735-8E05-BB9A00DDD58E}" name="Esito" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{62C11167-AB90-4C9D-AB96-CAA447BE5186}" name="Risultato ottenuto" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{0D1A1144-00D0-4FE6-A0D5-FFB26B983ADB}" name="Screenshot" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{3C60A41E-791B-4FAD-ADE1-BCB0D66A8574}" name="Note" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{EB876EC9-8950-4C9E-86BE-0FACA74E1014}" name="ID Test" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{EB9B5E9C-47F6-4F74-AAF0-EA51262287B5}" name="Area" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{52078D58-E160-4F5C-8E20-667269BD8E65}" name="Obiettivo" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{683810AF-1BE0-4D6F-9DB9-17FE773290C1}" name="Endpoint" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{9154901E-12A0-4767-BCFB-66395C70A786}" name="Metodo HTTP" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{C2F5DBF9-5AF1-4772-AC3D-C8C62175A99E}" name="Payload JSON" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{0E07DB66-29AC-4137-8446-4A4A24F26F1E}" name="Risultato atteso - Status Code" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{803671B0-E093-430D-967C-418EDDBE36A7}" name="Risultato atteso - Dettaglio" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{FB4642C7-35C4-4735-8E05-BB9A00DDD58E}" name="Esito" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{62C11167-AB90-4C9D-AB96-CAA447BE5186}" name="Risultato ottenuto" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{0D1A1144-00D0-4FE6-A0D5-FFB26B983ADB}" name="Screenshot" dataDxfId="19"/>
+    <tableColumn id="12" xr3:uid="{3C60A41E-791B-4FAD-ADE1-BCB0D66A8574}" name="Note" dataDxfId="18"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{24EE69B5-7BDF-4338-AD9C-BC1914DA8D01}" name="Table1342" displayName="Table1342" ref="A1:L27" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A1:L27" xr:uid="{A5FE12E1-30BD-4610-B2EA-DC3BCD910670}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{F161A8EE-6C0A-429C-8EDF-38BCE6A5C617}" name="ID Test" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{A4CC6D42-BD3E-411F-A782-E5E581E7C31D}" name="Area" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{C416FAE7-9B41-47F5-A86A-6069A3A9CA82}" name="Obiettivo" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{6AE2E0A7-A71C-43F2-8B7B-1D89210B70FC}" name="Endpoint" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{DCC71EE7-695B-4DA5-9E47-24EEC2066332}" name="Metodo HTTP" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{EF13877F-7D50-4B48-80E8-A77672DFAF22}" name="Payload JSON" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{DEBE20AF-9632-429C-8BF3-0CFC095DDAA1}" name="Risultato atteso - Status Code" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{33516315-38D4-4B89-9A05-FC8EA73F239D}" name="Risultato atteso - Dettaglio" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{CE3E1192-44C3-45E1-AE16-93214336C80F}" name="Esito" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{FE86ED33-8498-4516-8983-081D63D6E0E5}" name="Risultato ottenuto" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{E04D5FA0-F264-4042-BE1E-826BBF2E7575}" name="Screenshot" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{D7BF6AAF-EBF0-4133-A47D-E2E7FB9F02BB}" name="Note" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1504,7 +1570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86B77A02-D3E0-4056-A4CA-AF296B95BA61}">
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr defaultColWidth="31.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -1562,216 +1628,216 @@
     </row>
     <row r="2" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>164</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="D8" s="1" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>167</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>20</v>
@@ -1780,27 +1846,27 @@
         <v>21</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>168</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>20</v>
@@ -1809,172 +1875,172 @@
         <v>21</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>23</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>169</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="K12" s="1" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="K13" s="1" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>16</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>173</v>
+        <v>156</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="K15" s="1" t="s">
-        <v>174</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>25</v>
@@ -1983,27 +2049,27 @@
         <v>21</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>25</v>
@@ -2012,143 +2078,143 @@
         <v>21</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>23</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>176</v>
+        <v>159</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>177</v>
+        <v>160</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>22</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>178</v>
+        <v>161</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>16</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>179</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>19</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>180</v>
+        <v>163</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>13</v>
@@ -2166,18 +2232,18 @@
         <v>17</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>163</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>13</v>
@@ -2192,217 +2258,1035 @@
         <v>19</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>162</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>16</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>161</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>16</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>160</v>
+        <v>143</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>19</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>159</v>
+        <v>142</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="D27" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G27" s="1" t="s">
         <v>16</v>
       </c>
       <c r="H27" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="I2:I27">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+      <formula>"KO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I27" xr:uid="{F9FA5552-9B13-4186-A47D-1950B711ECD9}">
+      <formula1>"OK,KO"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A13C9FDD-A939-4DB4-9224-642B99CEC015}">
+  <dimension ref="A1:L27"/>
+  <sheetFormatPr defaultColWidth="31.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.42578125" style="1"/>
+    <col min="4" max="4" width="34.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.42578125" style="1"/>
+    <col min="7" max="7" width="30.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="31.42578125" style="1"/>
+    <col min="9" max="9" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="51.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="54.28515625" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="31.42578125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>120</v>
       </c>
+      <c r="B24" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>164</v>
+      </c>
       <c r="K27" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="75" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="75" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="90" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="K30" s="1" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I30">
+  <conditionalFormatting sqref="I2:I27">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
@@ -2411,7 +3295,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I30" xr:uid="{F9FA5552-9B13-4186-A47D-1950B711ECD9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I27" xr:uid="{91C71B9B-B0BE-466F-8E22-BD656A765F9F}">
       <formula1>"OK,KO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>